<commit_message>
Rewrite all 60 challenge scenarios and feedback copy in Excel
- Lighter, warmer language across Challenge Library
- Shorter statements, reflections, and Why Humans Do This fields
- Add rewrite-content.py for batch content updates
- Regenerate challenges.json from updated source

Co-authored-by: andreeanesu <andreeanesu@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/second-thought/data/source/cognitive_bias_trainer.xlsx
+++ b/second-thought/data/source/cognitive_bias_trainer.xlsx
@@ -1950,7 +1950,7 @@
       </c>
       <c r="D7" s="19" t="inlineStr">
         <is>
-          <t>In a job interview, the recruiter asks for a desired salary first, and the candidate's answer ends up anchoring the entire negotiation.</t>
+          <t>In a job interview, they ask for my salary first — and that number ends up anchoring the whole negotiation.</t>
         </is>
       </c>
       <c r="E7" s="19" t="inlineStr">
@@ -1980,17 +1980,17 @@
       </c>
       <c r="J7" s="19" t="inlineStr">
         <is>
-          <t>The number stated first becomes the reference point for the rest of the discussion, even as new information emerges.</t>
+          <t>The first number spoken becomes the reference for everything after.</t>
         </is>
       </c>
       <c r="K7" s="19" t="inlineStr">
         <is>
-          <t>Have you ever felt 'stuck' near a number you mentioned early in a conversation?</t>
+          <t>Have you ever felt stuck near a number you said early on?</t>
         </is>
       </c>
       <c r="L7" s="19" t="inlineStr">
         <is>
-          <t>Early numbers are hard to mentally let go of, even when new information suggests they should change.</t>
+          <t>Early numbers are hard to let go of — even when new info suggests we should move on.</t>
         </is>
       </c>
       <c r="M7" s="19" t="inlineStr">
@@ -2027,7 +2027,7 @@
       </c>
       <c r="D8" s="19" t="inlineStr">
         <is>
-          <t>After seeing several news stories about plane crashes, someone becomes afraid of flying, even though flying is statistically safer than driving.</t>
+          <t>After a few plane-crash stories in the news, flying feels terrifying — even though stats say driving is riskier.</t>
         </is>
       </c>
       <c r="E8" s="19" t="inlineStr">
@@ -2057,17 +2057,17 @@
       </c>
       <c r="J8" s="19" t="inlineStr">
         <is>
-          <t>Vivid, memorable news stories make plane crashes feel more common than they statistically are.</t>
+          <t>Vivid stories feel more common than they are.</t>
         </is>
       </c>
       <c r="K8" s="19" t="inlineStr">
         <is>
-          <t>Can you think of a fear you have that might be based on memorable stories rather than actual statistics?</t>
+          <t>Any fear you have that might come from memorable stories, not stats?</t>
         </is>
       </c>
       <c r="L8" s="19" t="inlineStr">
         <is>
-          <t>Our brains use ease of recall as a shortcut for judging probability.</t>
+          <t>Easy-to-recall events feel more likely. Our brain uses memory as a shortcut.</t>
         </is>
       </c>
       <c r="M8" s="19" t="inlineStr">
@@ -2104,7 +2104,7 @@
       </c>
       <c r="D9" s="19" t="inlineStr">
         <is>
-          <t>A parent refuses to vaccinate their child after reading a viral post about a rare side effect, while ignoring the far more common risks of the disease itself.</t>
+          <t>I saw one viral post about a rare vaccine side effect — and it stuck more than the disease risks I ignored.</t>
         </is>
       </c>
       <c r="E9" s="19" t="inlineStr">
@@ -2134,17 +2134,17 @@
       </c>
       <c r="J9" s="19" t="inlineStr">
         <is>
-          <t>A vivid, emotionally charged story is easier to recall than statistical data, distorting the perceived risk.</t>
+          <t>One vivid story outweighed the broader data.</t>
         </is>
       </c>
       <c r="K9" s="19" t="inlineStr">
         <is>
-          <t>When assessing a health risk, do you check the data or rely on the story that comes to mind first?</t>
+          <t>On health risks, do you check the data or trust the story that sticks?</t>
         </is>
       </c>
       <c r="L9" s="19" t="inlineStr">
         <is>
-          <t>Emotionally striking examples stick in memory far more than dry statistics.</t>
+          <t>Emotional stories lodge in memory. Dry statistics often don't.</t>
         </is>
       </c>
       <c r="M9" s="19" t="inlineStr">
@@ -2181,7 +2181,7 @@
       </c>
       <c r="D10" s="19" t="inlineStr">
         <is>
-          <t>After a friend's house is burgled, someone starts believing burglaries are common in their neighborhood, even though crime rates have been falling for years.</t>
+          <t>After a friend's house was burgled, burglaries suddenly feel common here — even though crime has been falling.</t>
         </is>
       </c>
       <c r="E10" s="19" t="inlineStr">
@@ -2211,17 +2211,17 @@
       </c>
       <c r="J10" s="19" t="inlineStr">
         <is>
-          <t>A single vivid, personal example outweighs broader statistical trends in shaping perceived risk.</t>
+          <t>One close story outweighed the wider trend.</t>
         </is>
       </c>
       <c r="K10" s="19" t="inlineStr">
         <is>
-          <t>Has a single story from someone you know ever changed how safe you feel, more than actual data would justify?</t>
+          <t>Has one person's story ever changed how safe you feel?</t>
         </is>
       </c>
       <c r="L10" s="19" t="inlineStr">
         <is>
-          <t>Personal, close-to-home stories feel more relevant and are recalled more easily than abstract statistics.</t>
+          <t>Stories from people we know feel real and relevant — more than numbers on a page.</t>
         </is>
       </c>
       <c r="M10" s="19" t="inlineStr">
@@ -2258,7 +2258,7 @@
       </c>
       <c r="D11" s="19" t="inlineStr">
         <is>
-          <t>A colleague is late to the meeting, and everyone assumes they're just lazy and disorganized, not knowing their car broke down that morning.</t>
+          <t>A colleague was late to the meeting. Everyone assumed they're lazy — not knowing their car broke down.</t>
         </is>
       </c>
       <c r="E11" s="19" t="inlineStr">
@@ -2288,17 +2288,17 @@
       </c>
       <c r="J11" s="19" t="inlineStr">
         <is>
-          <t>Observers default to a character-based explanation instead of considering the situation.</t>
+          <t>Character got blamed before circumstances were considered.</t>
         </is>
       </c>
       <c r="K11" s="19" t="inlineStr">
         <is>
-          <t>Next time someone is late, what situational reasons might explain it before you judge their character?</t>
+          <t>Next time someone's late — what situation might explain it?</t>
         </is>
       </c>
       <c r="L11" s="19" t="inlineStr">
         <is>
-          <t>We have limited information about others' circumstances, so we fill the gap with assumptions about their character.</t>
+          <t>We don't see others' full context, so we fill the gap with personality labels.</t>
         </is>
       </c>
       <c r="M11" s="19" t="inlineStr">
@@ -2335,7 +2335,7 @@
       </c>
       <c r="D12" s="19" t="inlineStr">
         <is>
-          <t>A driver cuts you off, and you immediately think 'what a reckless jerk,' without considering they might be rushing to an emergency.</t>
+          <t>Someone cut me off in traffic. I thought 'what a jerk' — without wondering if they had an emergency.</t>
         </is>
       </c>
       <c r="E12" s="19" t="inlineStr">
@@ -2365,17 +2365,17 @@
       </c>
       <c r="J12" s="19" t="inlineStr">
         <is>
-          <t>The behavior is attributed entirely to the other driver's character rather than a possible situational cause.</t>
+          <t>The action was blamed on character, not situation.</t>
         </is>
       </c>
       <c r="K12" s="19" t="inlineStr">
         <is>
-          <t>Have you ever driven aggressively because of your own circumstances that day?</t>
+          <t>Have you ever driven badly because of your own bad day?</t>
         </is>
       </c>
       <c r="L12" s="19" t="inlineStr">
         <is>
-          <t>It's easier to judge a stranger's character in an instant than to imagine their unseen situation.</t>
+          <t>It's faster to judge a stranger's character than imagine their unseen story.</t>
         </is>
       </c>
       <c r="M12" s="19" t="inlineStr">
@@ -2412,7 +2412,7 @@
       </c>
       <c r="D13" s="19" t="inlineStr">
         <is>
-          <t>A friend cancels plans last minute again, and you conclude they're unreliable, though it could also be a string of genuinely bad circumstances.</t>
+          <t>A friend cancelled last minute again. I decided they're unreliable — maybe it was just a run of bad luck.</t>
         </is>
       </c>
       <c r="E13" s="19" t="inlineStr">
@@ -2442,17 +2442,17 @@
       </c>
       <c r="J13" s="19" t="inlineStr">
         <is>
-          <t>A single explanation (character) is chosen quickly, when only the accumulation of many instances could clarify whether it's a real pattern.</t>
+          <t>One label stuck before a real pattern was clear.</t>
         </is>
       </c>
       <c r="K13" s="19" t="inlineStr">
         <is>
-          <t>How many times would something need to happen before you'd call it a pattern rather than bad luck?</t>
+          <t>How many times before you'd call something a pattern, not bad luck?</t>
         </is>
       </c>
       <c r="L13" s="19" t="inlineStr">
         <is>
-          <t>It's mentally efficient to settle on one clear explanation rather than track uncertainty over time.</t>
+          <t>One clear story feels easier than holding uncertainty over time.</t>
         </is>
       </c>
       <c r="M13" s="19" t="inlineStr">
@@ -2489,7 +2489,7 @@
       </c>
       <c r="D14" s="19" t="inlineStr">
         <is>
-          <t>A student says they passed the exam because they're smart, but failed the last one because the questions were unfair.</t>
+          <t>I passed because I'm smart — but failed last time because the questions were unfair.</t>
         </is>
       </c>
       <c r="E14" s="19" t="inlineStr">
@@ -2519,17 +2519,17 @@
       </c>
       <c r="J14" s="19" t="inlineStr">
         <is>
-          <t>Success is credited to personal ability while failure is blamed on external factors.</t>
+          <t>Success went to me; failure went to outside factors.</t>
         </is>
       </c>
       <c r="K14" s="19" t="inlineStr">
         <is>
-          <t>Think of your last success and failure - did you explain them the same way?</t>
+          <t>Your last win and loss — did you explain them the same way?</t>
         </is>
       </c>
       <c r="L14" s="19" t="inlineStr">
         <is>
-          <t>Crediting ourselves for success and blaming outside factors for failure protects our self-image.</t>
+          <t>Crediting ourselves for wins and blaming outside forces for losses protects how we feel about ourselves.</t>
         </is>
       </c>
       <c r="M14" s="19" t="inlineStr">
@@ -2566,7 +2566,7 @@
       </c>
       <c r="D15" s="19" t="inlineStr">
         <is>
-          <t>A team captain says the team won because of great strategy, but lost the next game because of a bad referee.</t>
+          <t>We won because of great strategy. We lost because of a bad referee.</t>
         </is>
       </c>
       <c r="E15" s="19" t="inlineStr">
@@ -2596,17 +2596,17 @@
       </c>
       <c r="J15" s="19" t="inlineStr">
         <is>
-          <t>The captain takes credit for the win but externalizes blame for the loss, rather than evaluating both fairly.</t>
+          <t>The win was ours; the loss was someone else's fault.</t>
         </is>
       </c>
       <c r="K15" s="19" t="inlineStr">
         <is>
-          <t>Can you recall a loss you blamed entirely on something outside your control?</t>
+          <t>A loss you blamed entirely on something outside your control?</t>
         </is>
       </c>
       <c r="L15" s="19" t="inlineStr">
         <is>
-          <t>Maintaining a positive self-image feels better than acknowledging personal shortcomings.</t>
+          <t>Keeping a positive self-image feels better than sitting with our own shortcomings.</t>
         </is>
       </c>
       <c r="M15" s="19" t="inlineStr">
@@ -2643,7 +2643,7 @@
       </c>
       <c r="D16" s="19" t="inlineStr">
         <is>
-          <t>A manager takes credit for a successful project but blames the team when a similar project fails, even though their own decisions played a role both times.</t>
+          <t>A manager took credit when a project worked — and blamed the team when a similar one failed.</t>
         </is>
       </c>
       <c r="E16" s="19" t="inlineStr">
@@ -2673,17 +2673,17 @@
       </c>
       <c r="J16" s="19" t="inlineStr">
         <is>
-          <t>Crediting success to oneself while shifting blame elsewhere for failure, even when personal decisions contributed to both, is a hallmark of self-serving bias.</t>
+          <t>Success was personal; failure was shifted away.</t>
         </is>
       </c>
       <c r="K16" s="19" t="inlineStr">
         <is>
-          <t>When a project you led fails, how much of the explanation do you attribute to yourself versus others?</t>
+          <t>When your project fails — how much do you own versus blame others?</t>
         </is>
       </c>
       <c r="L16" s="19" t="inlineStr">
         <is>
-          <t>Protecting our sense of competence is more comfortable than acknowledging shared responsibility for failure.</t>
+          <t>Protecting our sense of competence is easier than sharing responsibility for failure.</t>
         </is>
       </c>
       <c r="M16" s="19" t="inlineStr">
@@ -2720,7 +2720,7 @@
       </c>
       <c r="D17" s="19" t="inlineStr">
         <is>
-          <t>An investor keeps holding a failing stock because they've already put so much money into it, hoping it will recover.</t>
+          <t>I keep holding a failing stock because I've already put so much into it — hoping it'll bounce back.</t>
         </is>
       </c>
       <c r="E17" s="19" t="inlineStr">
@@ -2750,17 +2750,17 @@
       </c>
       <c r="J17" s="19" t="inlineStr">
         <is>
-          <t>The decision to keep holding is driven by past investment rather than the stock's future prospects.</t>
+          <t>Past money spent is driving the choice, not future prospects.</t>
         </is>
       </c>
       <c r="K17" s="19" t="inlineStr">
         <is>
-          <t>If you were deciding today with no prior investment, would you still choose to hold this stock?</t>
+          <t>If you were deciding fresh today, would you still hold it?</t>
         </is>
       </c>
       <c r="L17" s="19" t="inlineStr">
         <is>
-          <t>Admitting a past investment was a mistake feels like a loss, so we keep going to avoid that feeling.</t>
+          <t>Walking away feels like admitting a mistake. Staying avoids that pain — even when it costs more.</t>
         </is>
       </c>
       <c r="M17" s="19" t="inlineStr">
@@ -2797,7 +2797,7 @@
       </c>
       <c r="D18" s="19" t="inlineStr">
         <is>
-          <t>Someone stays in an unhappy relationship, thinking 'I've already spent five years on this, I can't leave now.'</t>
+          <t>I've spent five years in this relationship. I can't leave now — even though I'm unhappy.</t>
         </is>
       </c>
       <c r="E18" s="19" t="inlineStr">
@@ -2827,17 +2827,17 @@
       </c>
       <c r="J18" s="19" t="inlineStr">
         <is>
-          <t>Time already invested is treated as a reason to continue, even though it cannot be recovered either way.</t>
+          <t>Time already spent is treated as a reason to stay.</t>
         </is>
       </c>
       <c r="K18" s="19" t="inlineStr">
         <is>
-          <t>Would you enter this relationship today, knowing what you know now?</t>
+          <t>Would you start this relationship today, knowing what you know?</t>
         </is>
       </c>
       <c r="L18" s="19" t="inlineStr">
         <is>
-          <t>Walking away feels like admitting the time already spent was wasted, which is emotionally painful.</t>
+          <t>Leaving can feel like wasted years were wasted for nothing. That's painful.</t>
         </is>
       </c>
       <c r="M18" s="19" t="inlineStr">
@@ -2874,7 +2874,7 @@
       </c>
       <c r="D19" s="19" t="inlineStr">
         <is>
-          <t>A couple keeps eating an expensive, mediocre restaurant meal because they've already paid for it, even though they could stop.</t>
+          <t>We keep eating a mediocre meal we already paid for — even though we could stop.</t>
         </is>
       </c>
       <c r="E19" s="19" t="inlineStr">
@@ -2904,17 +2904,17 @@
       </c>
       <c r="J19" s="19" t="inlineStr">
         <is>
-          <t>The money already spent is gone regardless of whether they finish the meal, but it still shapes the decision to keep eating.</t>
+          <t>Money already spent shouldn't change whether we keep eating.</t>
         </is>
       </c>
       <c r="K19" s="19" t="inlineStr">
         <is>
-          <t>Does knowing you've already paid change how much you 'should' eat?</t>
+          <t>Does having paid change how much you 'should' finish?</t>
         </is>
       </c>
       <c r="L19" s="19" t="inlineStr">
         <is>
-          <t>We conflate the sunk cost with the ongoing decision, even when they're logically separate.</t>
+          <t>We mix up 'already spent' with 'what to do next' — even when they're separate decisions.</t>
         </is>
       </c>
       <c r="M19" s="19" t="inlineStr">
@@ -2951,7 +2951,7 @@
       </c>
       <c r="D20" s="19" t="inlineStr">
         <is>
-          <t>After a performance review with nine positive comments and one criticism, the employee can only think about the criticism all week.</t>
+          <t>Nine compliments and one criticism in my review — and I obsessed over the criticism all week.</t>
         </is>
       </c>
       <c r="E20" s="19" t="inlineStr">
@@ -2981,17 +2981,17 @@
       </c>
       <c r="J20" s="19" t="inlineStr">
         <is>
-          <t>The single negative comment outweighs the nine positive ones in the employee's mind, despite the imbalance in actual content.</t>
+          <t>One negative note outweighed nine positive ones.</t>
         </is>
       </c>
       <c r="K20" s="19" t="inlineStr">
         <is>
-          <t>After your last piece of feedback, did you remember the praise or the criticism more clearly?</t>
+          <t>Last feedback you got — praise or criticism stuck more?</t>
         </is>
       </c>
       <c r="L20" s="19" t="inlineStr">
         <is>
-          <t>Negative information historically signaled threats, so our brains evolved to prioritize it.</t>
+          <t>Bad news used to signal danger. Our brains still give it extra weight.</t>
         </is>
       </c>
       <c r="M20" s="19" t="inlineStr">
@@ -3028,7 +3028,7 @@
       </c>
       <c r="D21" s="19" t="inlineStr">
         <is>
-          <t>News outlets report far more negative stories than positive ones, because negative headlines get more clicks and attention.</t>
+          <t>News runs more bad stories than good ones — because negative headlines get more clicks.</t>
         </is>
       </c>
       <c r="E21" s="19" t="inlineStr">
@@ -3058,17 +3058,17 @@
       </c>
       <c r="J21" s="19" t="inlineStr">
         <is>
-          <t>Both audience attention and outlet incentives are shaped by our stronger response to negative information.</t>
+          <t>Outlets and audiences both lean toward negative news.</t>
         </is>
       </c>
       <c r="K21" s="19" t="inlineStr">
         <is>
-          <t>Do you click on negative headlines more often than positive ones?</t>
+          <t>Do you click negative headlines more than positive ones?</t>
         </is>
       </c>
       <c r="L21" s="19" t="inlineStr">
         <is>
-          <t>Our attention is drawn more strongly to potential threats or bad news than to good news.</t>
+          <t>Threats and bad news pull our attention harder than good news.</t>
         </is>
       </c>
       <c r="M21" s="19" t="inlineStr">
@@ -3105,7 +3105,7 @@
       </c>
       <c r="D22" s="19" t="inlineStr">
         <is>
-          <t>One critical comment from a partner can outweigh many compliments, even though the ratio of positive to negative comments has been high.</t>
+          <t>One critical comment from my partner stuck more than months of compliments.</t>
         </is>
       </c>
       <c r="E22" s="19" t="inlineStr">
@@ -3135,17 +3135,17 @@
       </c>
       <c r="J22" s="19" t="inlineStr">
         <is>
-          <t>A single negative remark can dominate emotional memory of a relationship, disproportionate to its actual frequency.</t>
+          <t>A single negative remark dominated the emotional memory.</t>
         </is>
       </c>
       <c r="K22" s="19" t="inlineStr">
         <is>
-          <t>Can you recall a relationship where one negative comment overshadowed months of positive ones?</t>
+          <t>One comment that overshadowed a lot of good moments?</t>
         </is>
       </c>
       <c r="L22" s="19" t="inlineStr">
         <is>
-          <t>Negative experiences are processed more deeply and remembered more vividly than positive ones.</t>
+          <t>Negative moments are processed more deeply and remembered more vividly.</t>
         </is>
       </c>
       <c r="M22" s="19" t="inlineStr">
@@ -3182,7 +3182,7 @@
       </c>
       <c r="D23" s="19" t="inlineStr">
         <is>
-          <t>A well-dressed, articulate job candidate is assumed to also be highly competent at the technical parts of the job, without evidence.</t>
+          <t>A polished, articulate candidate seemed competent at the technical work too — without any proof.</t>
         </is>
       </c>
       <c r="E23" s="19" t="inlineStr">
@@ -3212,17 +3212,17 @@
       </c>
       <c r="J23" s="19" t="inlineStr">
         <is>
-          <t>A positive impression in one area (presentation) spills over into an unjustified assumption about an unrelated area (technical skill).</t>
+          <t>A good impression in one area spilled into another.</t>
         </is>
       </c>
       <c r="K23" s="19" t="inlineStr">
         <is>
-          <t>Have you ever assumed someone was good at their job just because they seemed confident?</t>
+          <t>Assumed someone was good at their job because they seemed confident?</t>
         </is>
       </c>
       <c r="L23" s="19" t="inlineStr">
         <is>
-          <t>It's mentally efficient to form one overall impression rather than evaluate every trait separately.</t>
+          <t>One overall impression is easier than judging each skill separately.</t>
         </is>
       </c>
       <c r="M23" s="19" t="inlineStr">
@@ -3259,7 +3259,7 @@
       </c>
       <c r="D24" s="19" t="inlineStr">
         <is>
-          <t>A celebrity endorses a health product, and fans assume the product must be effective because they like the celebrity.</t>
+          <t>A celebrity endorsed a health product — so fans assumed it works, because they like the celebrity.</t>
         </is>
       </c>
       <c r="E24" s="19" t="inlineStr">
@@ -3289,17 +3289,17 @@
       </c>
       <c r="J24" s="19" t="inlineStr">
         <is>
-          <t>Positive feelings toward the celebrity transfer to an unrelated claim about the product's effectiveness.</t>
+          <t>Feelings about the person transferred to the product.</t>
         </is>
       </c>
       <c r="K24" s="19" t="inlineStr">
         <is>
-          <t>Would you trust this product's claims as much if a stranger, not a celebrity, made them?</t>
+          <t>Would you trust the claim as much from a stranger?</t>
         </is>
       </c>
       <c r="L24" s="19" t="inlineStr">
         <is>
-          <t>We transfer trust from people we like to things they're associated with.</t>
+          <t>We pass trust from people we like to things they're linked with.</t>
         </is>
       </c>
       <c r="M24" s="19" t="inlineStr">
@@ -3336,7 +3336,7 @@
       </c>
       <c r="D25" s="19" t="inlineStr">
         <is>
-          <t>A charismatic new colleague is quickly promoted, and people assume all their ideas must be good, even ones that haven't actually been tested.</t>
+          <t>A charismatic colleague got promoted fast — and people assumed all their ideas were good, untested ones included.</t>
         </is>
       </c>
       <c r="E25" s="19" t="inlineStr">
@@ -3366,7 +3366,7 @@
       </c>
       <c r="J25" s="19" t="inlineStr">
         <is>
-          <t>Likeability creates a general positive impression that extends, without evidence, to the quality of their ideas.</t>
+          <t>Likeability stretched to ideas without evidence.</t>
         </is>
       </c>
       <c r="K25" s="19" t="inlineStr">
@@ -3376,7 +3376,7 @@
       </c>
       <c r="L25" s="19" t="inlineStr">
         <is>
-          <t>A strong positive first impression is hard to update, even when specific evidence is missing.</t>
+          <t>A strong first impression is hard to update — even when proof is missing.</t>
         </is>
       </c>
       <c r="M25" s="19" t="inlineStr">
@@ -3413,7 +3413,7 @@
       </c>
       <c r="D26" s="19" t="inlineStr">
         <is>
-          <t>A new employee arrives late on their first day, and colleagues immediately assume they're unreliable and probably not very hardworking either.</t>
+          <t>A new hire was late on day one. Colleagues decided they're unreliable and probably not hardworking.</t>
         </is>
       </c>
       <c r="E26" s="19" t="inlineStr">
@@ -3443,17 +3443,17 @@
       </c>
       <c r="J26" s="19" t="inlineStr">
         <is>
-          <t>One negative trait (lateness) is generalized into unrelated negative assumptions about work ethic.</t>
+          <t>One slip became a whole personality judgment.</t>
         </is>
       </c>
       <c r="K26" s="19" t="inlineStr">
         <is>
-          <t>Has one early mistake ever colored how you saw someone's whole personality?</t>
+          <t>One early mistake that colored how you saw someone?</t>
         </is>
       </c>
       <c r="L26" s="19" t="inlineStr">
         <is>
-          <t>A single negative impression is mentally simplified into 'this person is generally bad' rather than staying specific.</t>
+          <t>One flaw gets simplified into 'this person is generally bad' instead of staying specific.</t>
         </is>
       </c>
       <c r="M26" s="19" t="inlineStr">
@@ -3490,7 +3490,7 @@
       </c>
       <c r="D27" s="19" t="inlineStr">
         <is>
-          <t>Someone mispronounces a word in a presentation, and the audience starts assuming they don't really know the topic well.</t>
+          <t>Someone mispronounced a word in a talk — and the audience doubted whether they know the topic at all.</t>
         </is>
       </c>
       <c r="E27" s="19" t="inlineStr">
@@ -3520,17 +3520,17 @@
       </c>
       <c r="J27" s="19" t="inlineStr">
         <is>
-          <t>A minor, unrelated slip is generalized into doubting the person's actual competence.</t>
+          <t>A small slip was stretched into a competence judgment.</t>
         </is>
       </c>
       <c r="K27" s="19" t="inlineStr">
         <is>
-          <t>Have you ever judged someone's expertise based on an unrelated small mistake?</t>
+          <t>Judged someone's expertise over an unrelated small mistake?</t>
         </is>
       </c>
       <c r="L27" s="19" t="inlineStr">
         <is>
-          <t>Our brain looks for a consistent story, and one flaw is used to build a broader negative narrative.</t>
+          <t>Our brain wants one consistent story — and one flaw builds a negative one fast.</t>
         </is>
       </c>
       <c r="M27" s="19" t="inlineStr">
@@ -3567,7 +3567,7 @@
       </c>
       <c r="D28" s="19" t="inlineStr">
         <is>
-          <t>A public figure makes one factual error in an interview, and viewers dismiss everything else they said, even the parts backed by solid evidence.</t>
+          <t>A public figure got one fact wrong — and viewers dismissed everything else they said, even the solid parts.</t>
         </is>
       </c>
       <c r="E28" s="19" t="inlineStr">
@@ -3597,17 +3597,17 @@
       </c>
       <c r="J28" s="19" t="inlineStr">
         <is>
-          <t>One mistake is generalized to discredit an entire body of otherwise well-supported claims.</t>
+          <t>One error discredited the whole message.</t>
         </is>
       </c>
       <c r="K28" s="19" t="inlineStr">
         <is>
-          <t>When someone makes one error, do you dismiss everything else they say?</t>
+          <t>When someone errs once, do you dismiss everything they say?</t>
         </is>
       </c>
       <c r="L28" s="19" t="inlineStr">
         <is>
-          <t>A single clear flaw feels like reliable evidence, even when it doesn't logically extend to everything else.</t>
+          <t>One clear mistake feels like reliable evidence — even when it isn't about everything else.</t>
         </is>
       </c>
       <c r="M28" s="19" t="inlineStr">
@@ -3644,7 +3644,7 @@
       </c>
       <c r="D29" s="19" t="inlineStr">
         <is>
-          <t>Business advice books focus on interviews with successful entrepreneurs, ignoring the far larger number who tried similar strategies and failed.</t>
+          <t>Success books interview winning entrepreneurs — not the many who tried the same thing and failed.</t>
         </is>
       </c>
       <c r="E29" s="19" t="inlineStr">
@@ -3674,17 +3674,17 @@
       </c>
       <c r="J29" s="19" t="inlineStr">
         <is>
-          <t>The sample only includes 'survivors' (successful entrepreneurs), so the strategies that seem to work may not actually be reliable.</t>
+          <t>We only hear from survivors, so strategies look more reliable than they are.</t>
         </is>
       </c>
       <c r="K29" s="19" t="inlineStr">
         <is>
-          <t>When you read a success story, do you ever ask how many people tried the same thing and failed?</t>
+          <t>Reading a success story — do you ask who tried the same and failed?</t>
         </is>
       </c>
       <c r="L29" s="19" t="inlineStr">
         <is>
-          <t>Failures are often less visible, less discussed, or simply invisible to us, so successes dominate our sample.</t>
+          <t>Failures are quieter, less visible, and less fun to talk about.</t>
         </is>
       </c>
       <c r="M29" s="19" t="inlineStr">
@@ -3721,7 +3721,7 @@
       </c>
       <c r="D30" s="19" t="inlineStr">
         <is>
-          <t>A magazine article claims 'these five habits made these CEOs successful,' without checking whether unsuccessful people had the same habits.</t>
+          <t>'These five habits made CEOs successful' — with no check on failed CEOs who had the same habits.</t>
         </is>
       </c>
       <c r="E30" s="19" t="inlineStr">
@@ -3751,17 +3751,17 @@
       </c>
       <c r="J30" s="19" t="inlineStr">
         <is>
-          <t>Without a comparison group of unsuccessful people, it's impossible to know if the habits are actually linked to success.</t>
+          <t>Without a comparison group, the link to success is shaky.</t>
         </is>
       </c>
       <c r="K30" s="19" t="inlineStr">
         <is>
-          <t>If you never asked who failed, could you really trust an explanation of who succeeded?</t>
+          <t>Without asking who failed, can you trust why someone succeeded?</t>
         </is>
       </c>
       <c r="L30" s="19" t="inlineStr">
         <is>
-          <t>Success stories are more visible, celebrated, and interesting to tell than the many quiet failures.</t>
+          <t>Success stories are celebrated. Quiet failures disappear from view.</t>
         </is>
       </c>
       <c r="M30" s="19" t="inlineStr">
@@ -3798,7 +3798,7 @@
       </c>
       <c r="D31" s="19" t="inlineStr">
         <is>
-          <t>A student assumes a course must be easy because everyone still enrolled speaks well of it, not realizing the people who struggled already dropped out.</t>
+          <t>Everyone still in the course says it's easy — but the people who struggled already dropped out.</t>
         </is>
       </c>
       <c r="E31" s="19" t="inlineStr">
@@ -3828,17 +3828,17 @@
       </c>
       <c r="J31" s="19" t="inlineStr">
         <is>
-          <t>Only those who stayed and can be asked provide feedback, while those who dropped out are missing from the sample.</t>
+          <t>Only survivors are in the sample you're hearing from.</t>
         </is>
       </c>
       <c r="K31" s="19" t="inlineStr">
         <is>
-          <t>Whose voices might be missing from the feedback you're hearing?</t>
+          <t>Whose voices might be missing from the feedback you hear?</t>
         </is>
       </c>
       <c r="L31" s="19" t="inlineStr">
         <is>
-          <t>We naturally only hear from the people still present, forgetting the process that filtered others out.</t>
+          <t>We hear from who's left — and forget who already walked away.</t>
         </is>
       </c>
       <c r="M31" s="19" t="inlineStr">
@@ -3875,7 +3875,7 @@
       </c>
       <c r="D32" s="19" t="inlineStr">
         <is>
-          <t>After a stock crashes, an investor says 'I knew that was going to happen,' even though they bought more shares the week before.</t>
+          <t>After a stock crashed, I said 'I knew that would happen' — though I'd bought more the week before.</t>
         </is>
       </c>
       <c r="E32" s="19" t="inlineStr">
@@ -3905,17 +3905,17 @@
       </c>
       <c r="J32" s="19" t="inlineStr">
         <is>
-          <t>The investor's memory of their own confidence has shifted to match the now-known outcome.</t>
+          <t>Memory of what we believed shifted to match the outcome.</t>
         </is>
       </c>
       <c r="K32" s="19" t="inlineStr">
         <is>
-          <t>Have you ever claimed you 'knew' something would happen, despite acting otherwise beforehand?</t>
+          <t>Claimed you 'knew' something — despite acting the opposite before?</t>
         </is>
       </c>
       <c r="L32" s="19" t="inlineStr">
         <is>
-          <t>Knowing an outcome makes it feel inevitable in hindsight, distorting our memory of our own uncertainty.</t>
+          <t>Once we know the ending, it feels inevitable — and our memory bends to match.</t>
         </is>
       </c>
       <c r="M32" s="19" t="inlineStr">
@@ -3952,7 +3952,7 @@
       </c>
       <c r="D33" s="19" t="inlineStr">
         <is>
-          <t>After their team loses, a fan insists 'I knew we'd lose,' despite confidently predicting a win to friends the day before.</t>
+          <t>After the loss, I insisted 'I knew we'd lose' — though I'd predicted a win the day before.</t>
         </is>
       </c>
       <c r="E33" s="19" t="inlineStr">
@@ -3982,17 +3982,17 @@
       </c>
       <c r="J33" s="19" t="inlineStr">
         <is>
-          <t>The fan's recollection of their own prediction has been rewritten to fit the actual outcome.</t>
+          <t>Recollection of the prediction was rewritten after the fact.</t>
         </is>
       </c>
       <c r="K33" s="19" t="inlineStr">
         <is>
-          <t>Could you find a written or spoken prediction you made, and compare it honestly to what you now claim you thought?</t>
+          <t>Could you find what you actually predicted — versus what you claim now?</t>
         </is>
       </c>
       <c r="L33" s="19" t="inlineStr">
         <is>
-          <t>Our brains reconstruct memories of past beliefs in a way that's consistent with what we now know.</t>
+          <t>We rebuild past beliefs to fit what we know now.</t>
         </is>
       </c>
       <c r="M33" s="19" t="inlineStr">
@@ -4029,7 +4029,7 @@
       </c>
       <c r="D34" s="19" t="inlineStr">
         <is>
-          <t>After a project fails, the team concludes 'the risks were obvious from the start,' even though nobody flagged them clearly during planning.</t>
+          <t>After a project failed, the team said 'the risks were obvious from the start' — though nobody flagged them in planning.</t>
         </is>
       </c>
       <c r="E34" s="19" t="inlineStr">
@@ -4059,17 +4059,17 @@
       </c>
       <c r="J34" s="19" t="inlineStr">
         <is>
-          <t>Once the failure is known, the risks seem obvious in retrospect, even though they weren't clearly identified beforehand.</t>
+          <t>Risks look obvious only after failure is known.</t>
         </is>
       </c>
       <c r="K34" s="19" t="inlineStr">
         <is>
-          <t>Were the 'obvious' risks actually written down anywhere before the outcome was known?</t>
+          <t>Were the 'obvious' risks written down before the outcome?</t>
         </is>
       </c>
       <c r="L34" s="19" t="inlineStr">
         <is>
-          <t>Knowing the outcome makes the path to it feel more predictable than it actually was.</t>
+          <t>Knowing how it ended makes the path feel more predictable than it was.</t>
         </is>
       </c>
       <c r="M34" s="19" t="inlineStr">
@@ -4106,7 +4106,7 @@
       </c>
       <c r="D35" s="19" t="inlineStr">
         <is>
-          <t>A voter assumes 'most people' agree with their political opinion, mostly because everyone in their social circle does.</t>
+          <t>I assume most people share my political view — because everyone in my circle does.</t>
         </is>
       </c>
       <c r="E35" s="19" t="inlineStr">
@@ -4136,17 +4136,17 @@
       </c>
       <c r="J35" s="19" t="inlineStr">
         <is>
-          <t>The person mistakes agreement within their own social circle for agreement across the wider population.</t>
+          <t>My bubble was mistaken for the whole population.</t>
         </is>
       </c>
       <c r="K35" s="19" t="inlineStr">
         <is>
-          <t>How would you actually find out if most people agree with you, beyond your own social circle?</t>
+          <t>How would you check if most people agree — beyond your circle?</t>
         </is>
       </c>
       <c r="L35" s="19" t="inlineStr">
         <is>
-          <t>We're surrounded mostly by people similar to us, so their opinions feel like 'everyone's' opinion.</t>
+          <t>We're surrounded by similar people, so their views feel like everyone's.</t>
         </is>
       </c>
       <c r="M35" s="19" t="inlineStr">
@@ -4183,7 +4183,7 @@
       </c>
       <c r="D36" s="19" t="inlineStr">
         <is>
-          <t>Someone posts a controversial opinion online and is shocked by the backlash, assuming beforehand that 'everyone thinks this.'</t>
+          <t>I posted a hot take online and got slammed — I'd assumed 'everyone thinks this.'</t>
         </is>
       </c>
       <c r="E36" s="19" t="inlineStr">
@@ -4213,17 +4213,17 @@
       </c>
       <c r="J36" s="19" t="inlineStr">
         <is>
-          <t>The poster overestimated how widely shared their opinion actually was, mistaking their own bubble for a general consensus.</t>
+          <t>My bubble felt like consensus.</t>
         </is>
       </c>
       <c r="K36" s="19" t="inlineStr">
         <is>
-          <t>Has an online reaction ever surprised you because you assumed your view was more common than it was?</t>
+          <t>Online backlash that surprised you because you thought your view was common?</t>
         </is>
       </c>
       <c r="L36" s="19" t="inlineStr">
         <is>
-          <t>Our own beliefs feel intuitively 'normal' to us, so we assume others share them by default.</t>
+          <t>Our own beliefs feel normal — so we assume others share them.</t>
         </is>
       </c>
       <c r="M36" s="19" t="inlineStr">
@@ -4260,7 +4260,7 @@
       </c>
       <c r="D37" s="19" t="inlineStr">
         <is>
-          <t>A manager assumes the whole team supports a new policy because the two people who spoke up in the meeting agreed with it.</t>
+          <t>Two people agreed in a meeting — so the manager assumed the whole team supports the policy.</t>
         </is>
       </c>
       <c r="E37" s="19" t="inlineStr">
@@ -4290,17 +4290,17 @@
       </c>
       <c r="J37" s="19" t="inlineStr">
         <is>
-          <t>A small, vocal sample is mistaken for the views of the entire team, when silence doesn't necessarily mean agreement.</t>
+          <t>A vocal few stood in for everyone.</t>
         </is>
       </c>
       <c r="K37" s="19" t="inlineStr">
         <is>
-          <t>When only a few people speak up in a meeting, what can you actually conclude about everyone else's opinion?</t>
+          <t>When few speak up — what can you really conclude about the rest?</t>
         </is>
       </c>
       <c r="L37" s="19" t="inlineStr">
         <is>
-          <t>Vocal agreement is easy to notice and remember, while silent disagreement is invisible.</t>
+          <t>Loud agreement is easy to notice. Silent disagreement is invisible.</t>
         </is>
       </c>
       <c r="M37" s="19" t="inlineStr">
@@ -4337,7 +4337,7 @@
       </c>
       <c r="D38" s="19" t="inlineStr">
         <is>
-          <t>A manager gives the benefit of the doubt to a mistake made by someone from their own department, but is harsher about the same mistake from another department.</t>
+          <t>Same mistake from my department gets a pass — from another department, it's a serious problem.</t>
         </is>
       </c>
       <c r="E38" s="19" t="inlineStr">
@@ -4367,17 +4367,17 @@
       </c>
       <c r="J38" s="19" t="inlineStr">
         <is>
-          <t>The same behavior is judged differently depending on whether the person belongs to the manager's own group.</t>
+          <t>Group membership changed how the mistake was judged.</t>
         </is>
       </c>
       <c r="K38" s="19" t="inlineStr">
         <is>
-          <t>Do you judge mistakes from people 'like you' more gently than mistakes from others?</t>
+          <t>Judge mistakes from 'your people' more gently than from others?</t>
         </is>
       </c>
       <c r="L38" s="19" t="inlineStr">
         <is>
-          <t>We instinctively extend more trust and leniency to people we perceive as part of our own group.</t>
+          <t>We extend more trust and leniency to people we see as 'us.'</t>
         </is>
       </c>
       <c r="M38" s="19" t="inlineStr">
@@ -4414,7 +4414,7 @@
       </c>
       <c r="D39" s="19" t="inlineStr">
         <is>
-          <t>A fan believes a foul by their own team's player was 'clearly accidental,' but the same foul by the opposing team is 'obviously dirty play.'</t>
+          <t>Our player's foul was accidental. Their player's identical foul was dirty play.</t>
         </is>
       </c>
       <c r="E39" s="19" t="inlineStr">
@@ -4444,17 +4444,17 @@
       </c>
       <c r="J39" s="19" t="inlineStr">
         <is>
-          <t>Identical behavior is interpreted more charitably when it comes from the fan's own group.</t>
+          <t>Same action, different story — depending on the team.</t>
         </is>
       </c>
       <c r="K39" s="19" t="inlineStr">
         <is>
-          <t>Would you interpret this action the same way if the team names were switched?</t>
+          <t>Would you see it the same way if the teams were swapped?</t>
         </is>
       </c>
       <c r="L39" s="19" t="inlineStr">
         <is>
-          <t>Group loyalty shapes how we interpret ambiguous actions, favoring our own side.</t>
+          <t>Loyalty shapes how we read ambiguous actions — we favor our side.</t>
         </is>
       </c>
       <c r="M39" s="19" t="inlineStr">
@@ -4491,7 +4491,7 @@
       </c>
       <c r="D40" s="19" t="inlineStr">
         <is>
-          <t>A voter excuses a scandal involving a politician from their own party, but is outraged by a similar scandal from the opposing party.</t>
+          <t>I excuse a scandal from my party — but I'm outraged by the same thing from the other side.</t>
         </is>
       </c>
       <c r="E40" s="19" t="inlineStr">
@@ -4521,17 +4521,17 @@
       </c>
       <c r="J40" s="19" t="inlineStr">
         <is>
-          <t>The same type of behavior receives very different moral judgment depending on group allegiance.</t>
+          <t>Group allegiance changed the moral judgment.</t>
         </is>
       </c>
       <c r="K40" s="19" t="inlineStr">
         <is>
-          <t>Would this behavior bother you as much if it came from 'your side' instead of the other?</t>
+          <t>Would this bother you as much from your own side?</t>
         </is>
       </c>
       <c r="L40" s="19" t="inlineStr">
         <is>
-          <t>Protecting the reputation of our own group feels like protecting part of our own identity.</t>
+          <t>Protecting our group's reputation can feel like protecting part of ourselves.</t>
         </is>
       </c>
       <c r="M40" s="19" t="inlineStr">
@@ -4568,7 +4568,7 @@
       </c>
       <c r="D41" s="19" t="inlineStr">
         <is>
-          <t>Someone from the marketing team assumes everyone in engineering thinks and acts the same way, while recognizing lots of different personalities within marketing.</t>
+          <t>Marketing sees lots of personalities in marketing — but assumes everyone in engineering is the same.</t>
         </is>
       </c>
       <c r="E41" s="19" t="inlineStr">
@@ -4598,17 +4598,17 @@
       </c>
       <c r="J41" s="19" t="inlineStr">
         <is>
-          <t>The person sees diversity within their own group but assumes uniformity in a group they're less familiar with.</t>
+          <t>Diversity inside my group; sameness assumed outside it.</t>
         </is>
       </c>
       <c r="K41" s="19" t="inlineStr">
         <is>
-          <t>Which groups do you know well enough to see as diverse, and which do you lump together?</t>
+          <t>Which groups do you see as diverse — and which do you lump together?</t>
         </is>
       </c>
       <c r="L41" s="19" t="inlineStr">
         <is>
-          <t>We have more detailed exposure to our own group's individuals, but only surface-level exposure to other groups.</t>
+          <t>We know individuals in our group. Other groups we only see from a distance.</t>
         </is>
       </c>
       <c r="M41" s="19" t="inlineStr">
@@ -4645,7 +4645,7 @@
       </c>
       <c r="D42" s="19" t="inlineStr">
         <is>
-          <t>A person who has never lived abroad assumes that people from a certain country 'all think the same way' about a political issue.</t>
+          <t>I've never lived there — but I'm sure people from that country all think the same on this issue.</t>
         </is>
       </c>
       <c r="E42" s="19" t="inlineStr">
@@ -4675,17 +4675,17 @@
       </c>
       <c r="J42" s="19" t="inlineStr">
         <is>
-          <t>Limited exposure leads to an oversimplified, uniform view of an entire nationality.</t>
+          <t>Limited exposure became a uniform stereotype.</t>
         </is>
       </c>
       <c r="K42" s="19" t="inlineStr">
         <is>
-          <t>How much direct exposure do you actually have to the group you're generalizing about?</t>
+          <t>How much real exposure do you have to the group you're generalizing?</t>
         </is>
       </c>
       <c r="L42" s="19" t="inlineStr">
         <is>
-          <t>With less detailed information about a group, our minds fill in the gaps with broad, simplified assumptions.</t>
+          <t>Less detail about a group means broader, simpler assumptions.</t>
         </is>
       </c>
       <c r="M42" s="19" t="inlineStr">
@@ -4722,7 +4722,7 @@
       </c>
       <c r="D43" s="19" t="inlineStr">
         <is>
-          <t>A news report describes 'young people today' as if they all share one attitude, even though the reporter would never describe their own generation so simply.</t>
+          <t>A headline says 'young people today' all think one way — but we'd never describe our own generation that simply.</t>
         </is>
       </c>
       <c r="E43" s="19" t="inlineStr">
@@ -4752,17 +4752,17 @@
       </c>
       <c r="J43" s="19" t="inlineStr">
         <is>
-          <t>A large, diverse group is flattened into a single stereotype, a pattern common in how media describes generations or nationalities.</t>
+          <t>A diverse group was flattened into one attitude.</t>
         </is>
       </c>
       <c r="K43" s="19" t="inlineStr">
         <is>
-          <t>Would you accept this level of generalization about a group you belong to?</t>
+          <t>Would you accept this generalization about a group you're in?</t>
         </is>
       </c>
       <c r="L43" s="19" t="inlineStr">
         <is>
-          <t>Broad categories are easier to write and think about than the messy diversity within a real population.</t>
+          <t>Big categories are easier to write and think about than real diversity.</t>
         </is>
       </c>
       <c r="M43" s="19" t="inlineStr">
@@ -4799,7 +4799,7 @@
       </c>
       <c r="D44" s="19" t="inlineStr">
         <is>
-          <t>A treatment described as having a '90% survival rate' sounds much more appealing than the same treatment described as having a '10% mortality rate.'</t>
+          <t>'90% survival rate' sounds great. '10% mortality rate' sounds scary. Same treatment.</t>
         </is>
       </c>
       <c r="E44" s="19" t="inlineStr">
@@ -4829,17 +4829,17 @@
       </c>
       <c r="J44" s="19" t="inlineStr">
         <is>
-          <t>Identical statistics feel very different depending on whether they're framed positively (survival) or negatively (mortality).</t>
+          <t>Identical stats, different emotional frame.</t>
         </is>
       </c>
       <c r="K44" s="19" t="inlineStr">
         <is>
-          <t>Can you think of a decision where the way information was worded changed how you felt about it?</t>
+          <t>A decision where wording changed how you felt?</t>
         </is>
       </c>
       <c r="L44" s="19" t="inlineStr">
         <is>
-          <t>We respond emotionally to the frame of information (gain vs. loss) before we process the literal numbers.</t>
+          <t>We react to gain vs loss framing before we sit with the numbers.</t>
         </is>
       </c>
       <c r="M44" s="19" t="inlineStr">
@@ -4876,7 +4876,7 @@
       </c>
       <c r="D45" s="19" t="inlineStr">
         <is>
-          <t>A product labeled '90% fat free' sells better than the identical product labeled '10% fat,' even though the nutritional content is exactly the same.</t>
+          <t>'90% fat free' sells better than '10% fat' — same product on the label.</t>
         </is>
       </c>
       <c r="E45" s="19" t="inlineStr">
@@ -4906,17 +4906,17 @@
       </c>
       <c r="J45" s="19" t="inlineStr">
         <is>
-          <t>The positive frame ('fat free') is more appealing than the equivalent negative frame ('fat'), despite describing the same product.</t>
+          <t>Positive wording beat equivalent negative wording.</t>
         </is>
       </c>
       <c r="K45" s="19" t="inlineStr">
         <is>
-          <t>Have you ever chosen a product because of how it was labeled, rather than its actual content?</t>
+          <t>Chosen a product because of the label, not the content?</t>
         </is>
       </c>
       <c r="L45" s="19" t="inlineStr">
         <is>
-          <t>Positive-sounding wording triggers a more favorable gut reaction, independent of the actual facts.</t>
+          <t>Positive-sounding words trigger a warmer gut reaction — facts aside.</t>
         </is>
       </c>
       <c r="M45" s="19" t="inlineStr">
@@ -4953,7 +4953,7 @@
       </c>
       <c r="D46" s="19" t="inlineStr">
         <is>
-          <t>A policy is described as saving '200 lives' by one side and 'failing to save 100 lives' by the other, based on the exact same statistical outcome.</t>
+          <t>One side says a policy saves 200 lives. The other says it fails to save 100 — same outcome, different frame.</t>
         </is>
       </c>
       <c r="E46" s="19" t="inlineStr">
@@ -4983,17 +4983,17 @@
       </c>
       <c r="J46" s="19" t="inlineStr">
         <is>
-          <t>Both descriptions can be mathematically consistent with the same data, but each frame triggers a different emotional reaction.</t>
+          <t>Same numbers, opposite emotional pull.</t>
         </is>
       </c>
       <c r="K46" s="19" t="inlineStr">
         <is>
-          <t>When you read policy statistics, do you check whether a gain-frame and loss-frame would describe the exact same numbers?</t>
+          <t>Do you flip the frame to see if the numbers still hold?</t>
         </is>
       </c>
       <c r="L46" s="19" t="inlineStr">
         <is>
-          <t>Political communicators intentionally choose the frame most likely to trigger a favorable emotional response.</t>
+          <t>Communicators pick the frame that triggers the feeling they want.</t>
         </is>
       </c>
       <c r="M46" s="19" t="inlineStr">
@@ -5030,7 +5030,7 @@
       </c>
       <c r="D47" s="19" t="inlineStr">
         <is>
-          <t>An investor feels far more upset about losing $1,000 than they feel happy about gaining $1,000, even though the amounts are identical.</t>
+          <t>Losing $1,000 hurts more than gaining $1,000 feels good — same amount.</t>
         </is>
       </c>
       <c r="E47" s="19" t="inlineStr">
@@ -5060,17 +5060,17 @@
       </c>
       <c r="J47" s="19" t="inlineStr">
         <is>
-          <t>The emotional weight of a loss is felt more intensely than an equivalent gain, a hallmark of loss aversion.</t>
+          <t>Losses weigh heavier than equal gains.</t>
         </is>
       </c>
       <c r="K47" s="19" t="inlineStr">
         <is>
-          <t>Would you take a coin-flip bet to win $100 or lose $100? Why or why not?</t>
+          <t>Would you take a 50/50 bet to win or lose $100?</t>
         </is>
       </c>
       <c r="L47" s="19" t="inlineStr">
         <is>
-          <t>Our brains evolved to prioritize avoiding threats (like losses) over seeking equivalent rewards.</t>
+          <t>Avoiding loss mattered more for survival than chasing equal rewards.</t>
         </is>
       </c>
       <c r="M47" s="19" t="inlineStr">
@@ -5107,7 +5107,7 @@
       </c>
       <c r="D48" s="19" t="inlineStr">
         <is>
-          <t>In a negotiation, a person fights harder to avoid giving up a benefit they already have than they would to gain a new benefit of the same value.</t>
+          <t>In a negotiation, I'll fight harder to keep what I have than to gain something new of equal value.</t>
         </is>
       </c>
       <c r="E48" s="19" t="inlineStr">
@@ -5137,17 +5137,17 @@
       </c>
       <c r="J48" s="19" t="inlineStr">
         <is>
-          <t>The prospect of losing an existing benefit feels worse than the prospect of gaining an equivalent new one.</t>
+          <t>Losing what we have feels worse than gaining the same amount.</t>
         </is>
       </c>
       <c r="K48" s="19" t="inlineStr">
         <is>
-          <t>In your last negotiation, were you fighting harder to keep something or to gain something new?</t>
+          <t>Last negotiation — fighting harder to keep or to gain?</t>
         </is>
       </c>
       <c r="L48" s="19" t="inlineStr">
         <is>
-          <t>Losses are felt roughly twice as intensely as equivalent gains, so we work harder to avoid them.</t>
+          <t>Losses are felt more intensely than equivalent gains — often about twice as much.</t>
         </is>
       </c>
       <c r="M48" s="19" t="inlineStr">
@@ -5184,7 +5184,7 @@
       </c>
       <c r="D49" s="19" t="inlineStr">
         <is>
-          <t>Someone keeps an unused gym membership because canceling it feels like 'losing' something, even though they never use it.</t>
+          <t>I keep a gym membership I never use — canceling feels like losing something.</t>
         </is>
       </c>
       <c r="E49" s="19" t="inlineStr">
@@ -5214,17 +5214,17 @@
       </c>
       <c r="J49" s="19" t="inlineStr">
         <is>
-          <t>The decision is driven by an aversion to the feeling of loss (canceling) rather than an objective evaluation of ongoing costs and benefits.</t>
+          <t>Avoiding the feeling of loss beats the logic of stopping payment.</t>
         </is>
       </c>
       <c r="K49" s="19" t="inlineStr">
         <is>
-          <t>Is keeping this thing actually giving you value, or does canceling it just feel like a loss?</t>
+          <t>Keeping something unused — value, or just fear of losing it?</t>
         </is>
       </c>
       <c r="L49" s="19" t="inlineStr">
         <is>
-          <t>The emotional discomfort of 'losing' something, even something unused, outweighs the logical case for letting it go.</t>
+          <t>'Losing' something — even unused — can outweigh the clear case for letting go.</t>
         </is>
       </c>
       <c r="M49" s="19" t="inlineStr">
@@ -5261,7 +5261,7 @@
       </c>
       <c r="D50" s="19" t="inlineStr">
         <is>
-          <t>A smoker believes they're less likely than other smokers to develop health problems, without any specific reason to think they're different.</t>
+          <t>I smoke but tell myself I'm less likely to get sick than other smokers — no real reason why.</t>
         </is>
       </c>
       <c r="E50" s="19" t="inlineStr">
@@ -5291,17 +5291,17 @@
       </c>
       <c r="J50" s="19" t="inlineStr">
         <is>
-          <t>The belief that 'it won't happen to me' isn't based on evidence, just a general tendency to underestimate personal risk.</t>
+          <t>'It won't happen to me' without evidence.</t>
         </is>
       </c>
       <c r="K50" s="19" t="inlineStr">
         <is>
-          <t>Can you think of a risk you've downplayed for yourself compared to how you'd judge it for someone else?</t>
+          <t>A risk you've downplayed for yourself but not for others?</t>
         </is>
       </c>
       <c r="L50" s="19" t="inlineStr">
         <is>
-          <t>Believing bad things are less likely to happen to us personally helps maintain motivation and reduce anxiety.</t>
+          <t>Believing we're the exception reduces anxiety and keeps us moving.</t>
         </is>
       </c>
       <c r="M50" s="19" t="inlineStr">
@@ -5338,7 +5338,7 @@
       </c>
       <c r="D51" s="19" t="inlineStr">
         <is>
-          <t>A team consistently estimates that projects will take less time than they actually do, despite a long history of projects running late.</t>
+          <t>We always estimate projects will finish early — despite a long history of running late.</t>
         </is>
       </c>
       <c r="E51" s="19" t="inlineStr">
@@ -5368,17 +5368,17 @@
       </c>
       <c r="J51" s="19" t="inlineStr">
         <is>
-          <t>Repeated past evidence of delays is ignored in favor of an overly hopeful estimate for the current project.</t>
+          <t>Past delays get ignored for a hopeful new estimate.</t>
         </is>
       </c>
       <c r="K51" s="19" t="inlineStr">
         <is>
-          <t>Does your team's planning account for the actual historical track record, or just this project's best-case scenario?</t>
+          <t>Does planning use real history — or just this project's best case?</t>
         </is>
       </c>
       <c r="L51" s="19" t="inlineStr">
         <is>
-          <t>We tend to imagine the best-case scenario for our own plans, discounting evidence of past setbacks.</t>
+          <t>We picture the best outcome for our own plans and discount past slip-ups.</t>
         </is>
       </c>
       <c r="M51" s="19" t="inlineStr">
@@ -5415,7 +5415,7 @@
       </c>
       <c r="D52" s="19" t="inlineStr">
         <is>
-          <t>Someone doesn't save for retirement because they assume they'll 'figure it out later,' expecting their future income to be higher than statistics suggest is likely.</t>
+          <t>I'm not saving for retirement — I'll 'figure it out later' and assume I'll earn more than stats suggest.</t>
         </is>
       </c>
       <c r="E52" s="19" t="inlineStr">
@@ -5445,17 +5445,17 @@
       </c>
       <c r="J52" s="19" t="inlineStr">
         <is>
-          <t>The assumption of a better-than-average future outcome, without specific evidence, reflects a general tendency to expect personal good fortune.</t>
+          <t>A rosier-than-average future assumed without proof.</t>
         </is>
       </c>
       <c r="K52" s="19" t="inlineStr">
         <is>
-          <t>Is your financial plan based on an average, realistic scenario, or a best-case one?</t>
+          <t>Is your plan based on realistic odds — or a hoped-for best case?</t>
         </is>
       </c>
       <c r="L52" s="19" t="inlineStr">
         <is>
-          <t>An optimistic view of the future feels more comfortable than confronting uncertain or difficult odds.</t>
+          <t>An optimistic future feels easier than facing uncertain odds.</t>
         </is>
       </c>
       <c r="M52" s="19" t="inlineStr">
@@ -5492,7 +5492,7 @@
       </c>
       <c r="D53" s="19" t="inlineStr">
         <is>
-          <t>An employee stays in the default retirement plan their company assigned, even though a slightly better plan is available with just one form to switch.</t>
+          <t>I stayed in my company's default retirement plan — even though a better one needed just one form.</t>
         </is>
       </c>
       <c r="E53" s="19" t="inlineStr">
@@ -5522,17 +5522,17 @@
       </c>
       <c r="J53" s="19" t="inlineStr">
         <is>
-          <t>The default option is chosen simply because it requires no action, not because it's actually the best choice.</t>
+          <t>No action beat a slightly better option.</t>
         </is>
       </c>
       <c r="K53" s="19" t="inlineStr">
         <is>
-          <t>Is there a 'default' choice in your life you've never actually reconsidered?</t>
+          <t>A default choice you've never actually reconsidered?</t>
         </is>
       </c>
       <c r="L53" s="19" t="inlineStr">
         <is>
-          <t>Sticking with the current option requires no effort or decision, so it becomes the path of least resistance.</t>
+          <t>Sticking with now takes no effort. Change takes a decision.</t>
         </is>
       </c>
       <c r="M53" s="19" t="inlineStr">
@@ -5569,7 +5569,7 @@
       </c>
       <c r="D54" s="19" t="inlineStr">
         <is>
-          <t>A company keeps using an outdated software system because switching feels risky, even though the new system would clearly save time and money.</t>
+          <t>We keep outdated software because switching feels risky — though the new system would clearly save time and money.</t>
         </is>
       </c>
       <c r="E54" s="19" t="inlineStr">
@@ -5599,17 +5599,17 @@
       </c>
       <c r="J54" s="19" t="inlineStr">
         <is>
-          <t>The comfort of the familiar system outweighs a rational cost-benefit analysis of switching.</t>
+          <t>Familiar beat a rational case for change.</t>
         </is>
       </c>
       <c r="K54" s="19" t="inlineStr">
         <is>
-          <t>What's something at work you keep doing 'because that's how it's always been done'?</t>
+          <t>Something at work you keep because 'that's how it's always been'?</t>
         </is>
       </c>
       <c r="L54" s="19" t="inlineStr">
         <is>
-          <t>Change involves uncertainty and effort, while staying the same feels safe and predictable.</t>
+          <t>Change means uncertainty. Staying put feels safe and predictable.</t>
         </is>
       </c>
       <c r="M54" s="19" t="inlineStr">
@@ -5646,7 +5646,7 @@
       </c>
       <c r="D55" s="19" t="inlineStr">
         <is>
-          <t>Someone keeps their phone's default settings for years, assuming the manufacturer must have picked the best options, without ever exploring alternatives.</t>
+          <t>I've kept my phone's default settings for years — assuming the manufacturer picked the best ones.</t>
         </is>
       </c>
       <c r="E55" s="19" t="inlineStr">
@@ -5676,17 +5676,17 @@
       </c>
       <c r="J55" s="19" t="inlineStr">
         <is>
-          <t>The default is treated as inherently correct, simply because changing it requires deliberate action.</t>
+          <t>Default was treated as best without checking.</t>
         </is>
       </c>
       <c r="K55" s="19" t="inlineStr">
         <is>
-          <t>What default settings have you never questioned, in any part of your life?</t>
+          <t>Default settings you've never questioned — phone, habits, anything?</t>
         </is>
       </c>
       <c r="L55" s="19" t="inlineStr">
         <is>
-          <t>Defaults feel like an implicit recommendation, and changing them requires extra mental effort.</t>
+          <t>Defaults feel like a recommendation. Changing them takes mental effort.</t>
         </is>
       </c>
       <c r="M55" s="19" t="inlineStr">
@@ -5723,7 +5723,7 @@
       </c>
       <c r="D56" s="19" t="inlineStr">
         <is>
-          <t>After a single online course, someone feels confident enough to call themselves an expert in a field that professionals spend years mastering.</t>
+          <t>After one online course, I felt like an expert in a field professionals study for years.</t>
         </is>
       </c>
       <c r="E56" s="19" t="inlineStr">
@@ -5753,17 +5753,17 @@
       </c>
       <c r="J56" s="19" t="inlineStr">
         <is>
-          <t>A small amount of knowledge creates a disproportionate sense of confidence, without the deeper understanding of what's still unknown.</t>
+          <t>A little learning created a lot of confidence.</t>
         </is>
       </c>
       <c r="K56" s="19" t="inlineStr">
         <is>
-          <t>Can you think of a skill where you felt confident early on, only to realize later how much you didn't know?</t>
+          <t>A skill where early confidence later met how much you didn't know?</t>
         </is>
       </c>
       <c r="L56" s="19" t="inlineStr">
         <is>
-          <t>Early learning often skips the part where you discover how much complexity still lies ahead.</t>
+          <t>Early learning skips the part where you discover how much is still ahead.</t>
         </is>
       </c>
       <c r="M56" s="19" t="inlineStr">
@@ -5800,7 +5800,7 @@
       </c>
       <c r="D57" s="19" t="inlineStr">
         <is>
-          <t>A beginner chess player is convinced they could beat a grandmaster with 'the right strategy,' underestimating just how much skill separates the two.</t>
+          <t>As a beginner, I'm sure I could beat a chess grandmaster with the right strategy.</t>
         </is>
       </c>
       <c r="E57" s="19" t="inlineStr">
@@ -5830,17 +5830,17 @@
       </c>
       <c r="J57" s="19" t="inlineStr">
         <is>
-          <t>Limited experience makes it hard to accurately judge the gap between beginner and expert skill levels.</t>
+          <t>Limited experience hid how wide the skill gap really is.</t>
         </is>
       </c>
       <c r="K57" s="19" t="inlineStr">
         <is>
-          <t>How do you usually find out how good you really are at something new?</t>
+          <t>How do you find out how good you really are at something new?</t>
         </is>
       </c>
       <c r="L57" s="19" t="inlineStr">
         <is>
-          <t>Without expert-level knowledge, it's hard to even recognize what expert-level skill looks like.</t>
+          <t>Without expert knowledge, it's hard to see what expert skill actually looks like.</t>
         </is>
       </c>
       <c r="M57" s="19" t="inlineStr">
@@ -5877,7 +5877,7 @@
       </c>
       <c r="D58" s="19" t="inlineStr">
         <is>
-          <t>Someone reads a few articles online and feels more confident diagnosing their symptoms than the doctor who has treated thousands of similar cases.</t>
+          <t>A few articles online — and I felt more sure about my symptoms than the doctor with thousands of cases.</t>
         </is>
       </c>
       <c r="E58" s="19" t="inlineStr">
@@ -5907,17 +5907,17 @@
       </c>
       <c r="J58" s="19" t="inlineStr">
         <is>
-          <t>A small amount of self-directed research can create a false sense of expertise compared to years of professional training.</t>
+          <t>Surface reading felt like real expertise.</t>
         </is>
       </c>
       <c r="K58" s="19" t="inlineStr">
         <is>
-          <t>How do you decide when your own research is enough, versus when you need expert input?</t>
+          <t>When is your own research enough — and when do you need a pro?</t>
         </is>
       </c>
       <c r="L58" s="19" t="inlineStr">
         <is>
-          <t>Surface-level information can feel complete, even when it's missing the depth that real expertise provides.</t>
+          <t>A little information can feel complete when depth is still missing.</t>
         </is>
       </c>
       <c r="M58" s="19" t="inlineStr">
@@ -5954,7 +5954,7 @@
       </c>
       <c r="D59" s="19" t="inlineStr">
         <is>
-          <t>A patient trusts a diet recommendation from a doctor, even when the doctor is recommending something outside their actual area of expertise.</t>
+          <t>I trusted a diet tip from my doctor — even though it wasn't their area of expertise.</t>
         </is>
       </c>
       <c r="E59" s="19" t="inlineStr">
@@ -5984,17 +5984,17 @@
       </c>
       <c r="J59" s="19" t="inlineStr">
         <is>
-          <t>The doctor's general authority is extended to a specific claim, even where their expertise may not directly apply.</t>
+          <t>General authority stretched to a specific claim.</t>
         </is>
       </c>
       <c r="K59" s="19" t="inlineStr">
         <is>
-          <t>Does the person's authority actually relate to the specific claim they're making?</t>
+          <t>Does their authority actually match this specific advice?</t>
         </is>
       </c>
       <c r="L59" s="19" t="inlineStr">
         <is>
-          <t>We use titles and status as mental shortcuts for trustworthiness, rather than evaluating each specific claim.</t>
+          <t>Titles and status become shortcuts for trust — instead of checking each claim.</t>
         </is>
       </c>
       <c r="M59" s="19" t="inlineStr">
@@ -6031,7 +6031,7 @@
       </c>
       <c r="D60" s="19" t="inlineStr">
         <is>
-          <t>A junior employee doesn't question a flawed plan because it came from a senior executive, assuming their seniority means the plan must be sound.</t>
+          <t>I didn't question a flawed plan because a senior executive proposed it.</t>
         </is>
       </c>
       <c r="E60" s="19" t="inlineStr">
@@ -6061,17 +6061,17 @@
       </c>
       <c r="J60" s="19" t="inlineStr">
         <is>
-          <t>The plan's merit is assumed based on the source's rank, rather than being evaluated on its own logic.</t>
+          <t>Rank stood in for a sound argument.</t>
         </is>
       </c>
       <c r="K60" s="19" t="inlineStr">
         <is>
-          <t>Have you ever gone along with an idea mainly because of who suggested it?</t>
+          <t>Gone along with an idea mainly because of who suggested it?</t>
         </is>
       </c>
       <c r="L60" s="19" t="inlineStr">
         <is>
-          <t>Deferring to authority feels safer and requires less individual scrutiny of the actual argument.</t>
+          <t>Deferring to authority feels safer than scrutinizing the idea itself.</t>
         </is>
       </c>
       <c r="M60" s="19" t="inlineStr">
@@ -6108,7 +6108,7 @@
       </c>
       <c r="D61" s="19" t="inlineStr">
         <is>
-          <t>An actor who played a doctor on television is invited to comment on a real medical topic, and viewers trust the opinion partly because of the actor's on-screen role.</t>
+          <t>An actor who played a doctor on TV comments on real medicine — and viewers partly trust them because of the role.</t>
         </is>
       </c>
       <c r="E61" s="19" t="inlineStr">
@@ -6138,17 +6138,17 @@
       </c>
       <c r="J61" s="19" t="inlineStr">
         <is>
-          <t>A perceived (fictional) authority transfers unearned credibility to a claim on a real, unrelated topic.</t>
+          <t>A fictional role lent unearned credibility.</t>
         </is>
       </c>
       <c r="K61" s="19" t="inlineStr">
         <is>
-          <t>Would you trust this opinion as much if you didn't know who was saying it?</t>
+          <t>Would you trust this take as much if you didn't know who was speaking?</t>
         </is>
       </c>
       <c r="L61" s="19" t="inlineStr">
         <is>
-          <t>Familiarity with someone in an authority-associated role can create a felt sense of expertise, even when it isn't real.</t>
+          <t>Familiarity with an authority-like role can feel like real expertise.</t>
         </is>
       </c>
       <c r="M61" s="19" t="inlineStr">

</xml_diff>

<commit_message>
Add tier start screen with per-tier progress tracking
- Add Tier column to Excel bias library and export to biases.json
- Start screen with 4 options: Tier 1, Tier 2, Tier 3, and Mix
- Track seen questions separately per tier in localStorage
- Show progress (seen/total) and bias count on each tier card
- Finish screen offers 'Choose another level' to return to picker
- Migrate legacy mix progress from old seen-challenges key

Co-authored-by: andreeanesu <andreeanesu@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/second-thought/data/source/cognitive_bias_trainer.xlsx
+++ b/second-thought/data/source/cognitive_bias_trainer.xlsx
@@ -648,7 +648,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="11" min="1" max="1"/>
@@ -696,6 +696,11 @@
           <t>Common Contexts</t>
         </is>
       </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Tier</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="60" customHeight="1" s="12">
       <c r="A2" s="19" t="inlineStr">
@@ -733,6 +738,9 @@
           <t>Politics, Investing, Relationships, News, Health, Social Media</t>
         </is>
       </c>
+      <c r="H2" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="3" ht="60" customHeight="1" s="12">
       <c r="A3" s="19" t="inlineStr">
@@ -770,6 +778,9 @@
           <t>Negotiation, Shopping, Salary discussions, Real estate, Everyday life</t>
         </is>
       </c>
+      <c r="H3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="4" ht="60" customHeight="1" s="12">
       <c r="A4" s="19" t="inlineStr">
@@ -807,6 +818,9 @@
           <t>Media, Health, Safety, Everyday life, News</t>
         </is>
       </c>
+      <c r="H4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="5" ht="60" customHeight="1" s="12">
       <c r="A5" s="19" t="inlineStr">
@@ -844,6 +858,9 @@
           <t>Work, Relationships, Driving, Social situations</t>
         </is>
       </c>
+      <c r="H5" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="6" ht="60" customHeight="1" s="12">
       <c r="A6" s="19" t="inlineStr">
@@ -881,6 +898,9 @@
           <t>Work, Sport, Academics, Relationships</t>
         </is>
       </c>
+      <c r="H6" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="7" ht="60" customHeight="1" s="12">
       <c r="A7" s="19" t="inlineStr">
@@ -918,6 +938,9 @@
           <t>Finance, Relationships, Work, Everyday life</t>
         </is>
       </c>
+      <c r="H7" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="8" ht="60" customHeight="1" s="12">
       <c r="A8" s="19" t="inlineStr">
@@ -955,6 +978,9 @@
           <t>Work, Relationships, Media, Self-awareness</t>
         </is>
       </c>
+      <c r="H8" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="9" ht="60" customHeight="1" s="12">
       <c r="A9" s="19" t="inlineStr">
@@ -992,6 +1018,9 @@
           <t>Work, Media, Social situations, Politics</t>
         </is>
       </c>
+      <c r="H9" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="10" ht="60" customHeight="1" s="12">
       <c r="A10" s="19" t="inlineStr">
@@ -1029,6 +1058,9 @@
           <t>Work, Social situations, Media</t>
         </is>
       </c>
+      <c r="H10" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="11" ht="60" customHeight="1" s="12">
       <c r="A11" s="19" t="inlineStr">
@@ -1066,6 +1098,9 @@
           <t>Work, Media, Finance, Learning</t>
         </is>
       </c>
+      <c r="H11" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="12" ht="60" customHeight="1" s="12">
       <c r="A12" s="19" t="inlineStr">
@@ -1103,6 +1138,9 @@
           <t>Finance, Sport, Politics, Work</t>
         </is>
       </c>
+      <c r="H12" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="13" ht="60" customHeight="1" s="12">
       <c r="A13" s="19" t="inlineStr">
@@ -1140,6 +1178,9 @@
           <t>Politics, Social Media, Work, Everyday life</t>
         </is>
       </c>
+      <c r="H13" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="14" ht="60" customHeight="1" s="12">
       <c r="A14" s="19" t="inlineStr">
@@ -1177,6 +1218,9 @@
           <t>Work, Politics, Sport, Social situations</t>
         </is>
       </c>
+      <c r="H14" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="15" ht="60" customHeight="1" s="12">
       <c r="A15" s="19" t="inlineStr">
@@ -1214,6 +1258,9 @@
           <t>Work, Social situations, Politics, Media</t>
         </is>
       </c>
+      <c r="H15" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="16" ht="60" customHeight="1" s="12">
       <c r="A16" s="19" t="inlineStr">
@@ -1251,6 +1298,9 @@
           <t>Health, Finance, Marketing, Politics</t>
         </is>
       </c>
+      <c r="H16" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="17" ht="60" customHeight="1" s="12">
       <c r="A17" s="19" t="inlineStr">
@@ -1288,6 +1338,9 @@
           <t>Finance, Negotiation, Everyday life, Work</t>
         </is>
       </c>
+      <c r="H17" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="18" ht="60" customHeight="1" s="12">
       <c r="A18" s="19" t="inlineStr">
@@ -1325,6 +1378,9 @@
           <t>Health, Finance, Work, Everyday life</t>
         </is>
       </c>
+      <c r="H18" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="19" ht="60" customHeight="1" s="12">
       <c r="A19" s="19" t="inlineStr">
@@ -1362,6 +1418,9 @@
           <t>Work, Finance, Everyday life, Politics</t>
         </is>
       </c>
+      <c r="H19" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="20" ht="60" customHeight="1" s="12">
       <c r="A20" s="19" t="inlineStr">
@@ -1399,6 +1458,9 @@
           <t>Work, Learning, Everyday life, Health</t>
         </is>
       </c>
+      <c r="H20" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="21" ht="60" customHeight="1" s="12">
       <c r="A21" s="19" t="inlineStr">
@@ -1435,6 +1497,9 @@
         <is>
           <t>Work, Health, Media, Politics</t>
         </is>
+      </c>
+      <c r="H21" t="n">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>